<commit_message>
Added new RDF data schemes and visual schemes for environment-table45-46, and fixed XLSX spreadsheet for environment-table45
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table45.xlsx
+++ b/sources/table_normalization/xlsx/environment-table45.xlsx
@@ -174,7 +174,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -182,16 +182,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -685,15 +683,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -717,7 +715,7 @@
       <c r="M2" s="1"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="10"/>
+      <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
@@ -736,16 +734,16 @@
       <c r="G3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="L3" s="1"/>
@@ -894,15 +892,15 @@
       <c r="M7" s="1"/>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -926,7 +924,7 @@
       <c r="M10" s="3"/>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="9"/>
+      <c r="A11" s="3"/>
       <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
@@ -945,16 +943,16 @@
       <c r="G11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="I11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="J11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="K11" s="6" t="s">
         <v>10</v>
       </c>
       <c r="L11" s="3"/>

</xml_diff>